<commit_message>
Populate character library from filled Excel tables
</commit_message>
<xml_diff>
--- a/library/01_Wuthering_Waves.xlsx
+++ b/library/01_Wuthering_Waves.xlsx
@@ -7,11 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wuthering Waves" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wuthering Waves'!$A$1:$D$1</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -415,14 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -446,8 +437,1185 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Sigrika</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Aero</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Luuk Herssen</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Spectro</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mornye</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roccia</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Havoc</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Lynae</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Spectro</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Aalto</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Aero</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Augusta</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Electro</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Baizhi</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Glacio</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Buling</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Electro</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Brant</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1.11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Camellya</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Havoc</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1.12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Cantarella</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Havoc</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Carlotta</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Glacio</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1.14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Changli</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1.15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Shorekeeper</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Spectro</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1.16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Lumi</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Electro</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1.17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Phoebe</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Spectro</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Xiangli Yao</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Electro</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1.19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Youhu</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Glacio</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1.20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Zani</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Spectro</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1.21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Zhezhi</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Glacio</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1.22</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Cartethyia</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Aero</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1.23</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Chisa</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Havoc</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1.24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Chixia</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1.25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Ciaccona</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Aero</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1.26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Danjin</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Havoc</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1.27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Denia</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1.28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Encore</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1.29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Galbrena</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>1.30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Hiyuki</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Glacio</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>1.31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Hsin</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Iuno</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Aero</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>1.33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Jianxin</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Aero</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>1.34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Jinhsi</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Spectro</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>1.35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Jingran</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>1.36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Jiyan</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Aero</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>1.37</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Lingyang</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Glacio</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>1.38</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Lupa</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>1.39</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Lucy</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Spectro</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>1.40</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Aemeath</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>1.41</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Mortefi</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Phrolova</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Havoc</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Qiuyuan</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Aero</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>1.44</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Qingxiao</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Aero</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>1.45</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Rebecca</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Electro</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Sanhua</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Glacio</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>1.47</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Suisui</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Glacio</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>1.48</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Suoming</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>1.49</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Taoqi</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Havoc</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Verina</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Spectro</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>1.51</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Yangyang</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Aero</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>1.52</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Yangyang: Xuanling</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Havoc</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>1.53</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Yinlin</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Electro</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Yuanwu</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Electro</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>